<commit_message>
Say in Dataset S2 that mantle lithosphere is excluded too
The total already left it out, since it is computed from the two columns the
sheet prints. The Read me now names it alongside serpentinite and organic
carbon, and gives the reason - mantle-derived carbon returning to the mantle is
not a sink of surface carbon - so the difference from the model's total_influx
is accounted for rather than unexplained.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GG6eoxS3E2hq56pSKk2b7G
</commit_message>
<xml_diff>
--- a/supplementary/Supplementary_Dataset_S2_carbon_model.xlsx
+++ b/supplementary/Supplementary_Dataset_S2_carbon_model.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A32"/>
+  <dimension ref="A1:A33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="118" customWidth="1" min="1" max="1"/>
@@ -585,67 +585,74 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">    their sum. Serpentinite carbon is mantle-derived and returns to the mantle rather than</t>
+          <t xml:space="preserve">    their sum. Serpentinite and mantle lithosphere carbon are mantle-derived and return to the</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">    representing a sink of surface carbon, so it is excluded, as is organic carbon; neither</t>
+          <t xml:space="preserve">    mantle rather than representing a sink of surface carbon, so both are excluded, as is</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">    enters the attribution behind Figure 4.</t>
+          <t xml:space="preserve">    organic carbon. None of the three enters the attribution behind Figure 4, whose</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr"/>
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    biological sink is pelagic sediment plus altered oceanic crust.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>Sources (files in the CCD_workflow_clean repository, steps/step10_carbon_cycle_degassing/</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>Alfonso_etal_2024_DM26/Outputs):</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">  • Atmospheric outflux: Notebook05/csv/05_atmospheric_influx_all_sources.csv</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">  • Plate influx: Notebook02/csv/02_plate_influx.csv</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">  • Net flux: Notebook05/csv/05_net_carbon_outflux.csv</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr"/>
-    </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="A32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>See the Provenance sheet for the exact files used and when they were last written.</t>
         </is>
@@ -20551,7 +20558,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-09-16 07:05 by Paper/make_supplementary_datasets.py. Rerun that script after any change to the workflow so these numbers stay in step with the analysis.</t>
+          <t>Generated 2026-09-16 07:07 by Paper/make_supplementary_datasets.py. Rerun that script after any change to the workflow so these numbers stay in step with the analysis.</t>
         </is>
       </c>
     </row>

</xml_diff>